<commit_message>
added surefire plug in pom file-14 may 2026
</commit_message>
<xml_diff>
--- a/src/test/resources/voterData.xlsx
+++ b/src/test/resources/voterData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aishw\Purushoth projects\Selenium Java Basics\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aishw\PurushothProjects\selenium-voter-automation\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CEBB494-C77C-4622-A887-D78D9766AED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15DC574D-26E9-4017-8298-AE896717C3F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Voter ID</t>
   </si>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="11.44140625"/>
@@ -433,20 +433,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s" s="0">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s" s="0">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s" s="0">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s" s="0">
-        <v>7</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>